<commit_message>
Updated metabolite additions of gastrin
</commit_message>
<xml_diff>
--- a/Tasks/Task_706_Gastrin_synthesis/metabolites_additions.xlsx
+++ b/Tasks/Task_706_Gastrin_synthesis/metabolites_additions.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Desktop\Project Papers to Pathways\MSP_p3_2026_hormone_cytokine_task_creation\Tasks\Task_704_ACTH_synthesis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Desktop\Project Papers to Pathways\MSP_p3_2026_hormone_cytokine_task_creation\Tasks\Task_706_Gastrin_synthesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB0D34C6-D5DD-4311-B7DE-F866C96EC753}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F73AF981-065D-48D5-94C6-A4BC23EE05D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CD5DF94A-FED4-4ED9-B2C5-1CBFE42F25CF}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="96">
   <si>
     <t>action</t>
   </si>
@@ -219,92 +219,119 @@
     <t>NADH[x]</t>
   </si>
   <si>
-    <t>pre-pro-opiomelanocortin-1[c]</t>
-  </si>
-  <si>
     <t>c</t>
   </si>
   <si>
     <t>gene-pseudo-metabolite</t>
   </si>
   <si>
-    <t>pre-pro-opiomelanocortin-2[c]</t>
-  </si>
-  <si>
-    <t>pre-pro-opiomelanocortin-2-SRP[c]</t>
-  </si>
-  <si>
     <t>gene-pseudo-metabolite-intermidiate</t>
   </si>
   <si>
-    <t>pre-pro-opiomelanocortin-2-SRP[t]</t>
-  </si>
-  <si>
     <t>t</t>
   </si>
   <si>
     <t>gene-pseudo-metabolite-intermediate</t>
   </si>
   <si>
-    <t>pre-pro-opiomelanocortin-2-SRP[r]</t>
-  </si>
-  <si>
     <t>r</t>
   </si>
   <si>
-    <t>pro-opiomelanocortin-2-SRP[r]</t>
-  </si>
-  <si>
-    <t>MPRSCCSRSGALLLALLLQASMEVRGWCLESSQCQDLTTESNLLECIRACKPDLSAETPMFPGNGDEQPLTENPRKYVMGHFRWDRFGRRNSSSSGSSGAGQKREDVSAGEDCGPLPEGGPEPRSDGAKPGPREGKRSYSMEHFRWGKPVGKKRRPVKVYPNGAEDESAEAFPLEFKRELTGQRLREGDGPDGPADDGAGAQADLEHSLLVAAEKKDEGPYRMEHFRWGSPPKDKRYGGFMTSEKSQTPLVTLFKNAIIKNAYKKGE</t>
-  </si>
-  <si>
     <t>P01189</t>
   </si>
   <si>
-    <t>ENSG00000115138</t>
-  </si>
-  <si>
-    <t>pomc-signal-peptide[r]</t>
-  </si>
-  <si>
-    <t>ERO1-4SH[r]</t>
-  </si>
-  <si>
-    <t>enzyme-metaboltie</t>
-  </si>
-  <si>
-    <t>ERO1-4S[r]</t>
-  </si>
-  <si>
-    <t>PDIA1-4SH[r]</t>
-  </si>
-  <si>
-    <t>PDIA1-4S[r]</t>
-  </si>
-  <si>
-    <t>pro-opiomelanocortin-2-SRP-oxidized-folded[r]</t>
-  </si>
-  <si>
-    <t>pro-ACTH</t>
-  </si>
-  <si>
     <t>mg</t>
   </si>
   <si>
-    <t>ACTH</t>
-  </si>
-  <si>
-    <t>MCEEETTALVCDNGSGLCKAGFAGDDAPRAVFPSIVGRPRHQGVMVGMGQKDSYVGDEAQSKRGILTLKYPIEHGIITNWDDMEKIWHHSFYNELRVAPEEHPTLLTEAPLNPKANREKMTQIMFETFNVPAMYVAIQAVLSLYASGRTTGIVLDSGDGVTHNVPIYEGYALPHAIMRLDLAGRDLTDYLMKILTERGYSFVTTAEREIVRDIKEKLCYVALDFENEMATAASSSSLEKSYELPDGQVITIGNERFRCPETLFQPSFIGMESAGIHETTYNSIMKCDIDIRKDLYANNVLSGGTTMYPGIADRMQKEITALAPSTMKIKIIAPPERKYSVWIGGSILASLSTFQQMWISKPEYDEAGPSIVHRKCF</t>
-  </si>
-  <si>
     <t>P63267</t>
+  </si>
+  <si>
+    <t>pre-pro-gastrin-1[c]</t>
+  </si>
+  <si>
+    <t>MQRLCVYVLIFALALAAFSEASWKPRSQQPDAPLGTGANRDLELPWLEQQGPASHHRRQLGPQGPPHLVADPSKKQGPWLEEEEEAYGWMDFGRRSAEDEN</t>
+  </si>
+  <si>
+    <t>P01350</t>
+  </si>
+  <si>
+    <t>ENSG00000184502</t>
+  </si>
+  <si>
+    <t>pre-pro-gastrin-2[c]</t>
+  </si>
+  <si>
+    <t>pre-pro-gastrin-2-SRP[c]</t>
+  </si>
+  <si>
+    <t>pre-pro-gastrin-2-SRP[t]</t>
+  </si>
+  <si>
+    <t>pre-pro-gastrin-2-SRP[r]</t>
+  </si>
+  <si>
+    <t>pro-gastrin-2-SRP[r]</t>
+  </si>
+  <si>
+    <t>pro-gastrin-signal-peptide[r]</t>
+  </si>
+  <si>
+    <t>MQRLCVYVLIFALALAAFSEA</t>
+  </si>
+  <si>
+    <t>pro-gastrin-2-sulfated [g]</t>
+  </si>
+  <si>
+    <t>g</t>
+  </si>
+  <si>
+    <t>pro-gastrin-2-sulfated-phosphorylated [g]</t>
+  </si>
+  <si>
+    <t>73-74-progastrin [ig]</t>
+  </si>
+  <si>
+    <t>[ig]</t>
+  </si>
+  <si>
+    <t>ig</t>
+  </si>
+  <si>
+    <t>C-peptide</t>
+  </si>
+  <si>
+    <t>AEDEN</t>
+  </si>
+  <si>
+    <t>36-37-Gastrin71-Gly [ig]</t>
+  </si>
+  <si>
+    <t>53-54-Gastrin34-Gly [mg</t>
+  </si>
+  <si>
+    <t>[mg]</t>
+  </si>
+  <si>
+    <t>Gastrin34-amide [mg]</t>
+  </si>
+  <si>
+    <t>MQRLCVYVLIFALALAAFSEASWKPRSQQPDAPLGTGANRDLELPWLEQQGPASHHRRQLGPQGPPHLVADPSKKQGPWLEEEEEAYGWMDFGRRS</t>
+  </si>
+  <si>
+    <t>Gastrin17-amide [mg]</t>
+  </si>
+  <si>
+    <t>Uniprot</t>
+  </si>
+  <si>
+    <t>Ensembl</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -351,6 +378,13 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -393,7 +427,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -422,6 +456,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -939,62 +979,80 @@
       <c r="L1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="13" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="N1" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="O1" s="13" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H2" s="6" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="I2" s="7"/>
       <c r="J2" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="K2" s="7"/>
+        <v>60</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>70</v>
+      </c>
       <c r="L2" s="9">
         <v>0</v>
       </c>
-      <c r="M2" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="N2" s="7"/>
-      <c r="O2" s="7"/>
+      <c r="M2" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="N2" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>72</v>
+      </c>
       <c r="P2" s="7"/>
     </row>
-    <row r="3" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H3" s="6" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="I3" s="7"/>
       <c r="J3" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="K3" s="7"/>
+        <v>60</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>70</v>
+      </c>
       <c r="L3" s="9">
         <v>0</v>
       </c>
-      <c r="M3" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="N3" s="7"/>
-      <c r="O3" s="7"/>
+      <c r="M3" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>72</v>
+      </c>
       <c r="P3" s="7"/>
     </row>
     <row r="4" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H4" s="6" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="I4" s="7"/>
       <c r="J4" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K4" s="7"/>
       <c r="L4" s="9">
         <v>0</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
@@ -1002,18 +1060,18 @@
     </row>
     <row r="5" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H5" s="6" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="I5" s="7"/>
       <c r="J5" s="8" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="K5" s="7"/>
       <c r="L5" s="9">
         <v>0</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
@@ -1021,100 +1079,98 @@
     </row>
     <row r="6" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H6" s="6" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="I6" s="7"/>
       <c r="J6" s="8" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="K6" s="7"/>
       <c r="L6" s="9">
         <v>0</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="N6" s="7"/>
       <c r="O6" s="7"/>
       <c r="P6" s="7"/>
     </row>
-    <row r="7" spans="1:16" ht="331.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H7" s="10" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="I7" s="7"/>
       <c r="J7" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="K7" s="8" t="s">
-        <v>72</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="K7" s="7"/>
       <c r="L7" s="9">
         <v>0</v>
       </c>
       <c r="M7" s="8" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="N7" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="O7" s="6" t="s">
-        <v>74</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="O7" s="7"/>
       <c r="P7" s="7"/>
     </row>
-    <row r="8" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H8" s="10" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I8" s="7"/>
       <c r="J8" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="K8" s="7"/>
+        <v>65</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>79</v>
+      </c>
       <c r="L8" s="9">
         <v>0</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
     </row>
     <row r="9" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="H9" s="8" t="s">
-        <v>76</v>
+      <c r="H9" s="6" t="s">
+        <v>80</v>
       </c>
       <c r="I9" s="7"/>
       <c r="J9" s="8" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="K9" s="7"/>
       <c r="L9" s="9">
         <v>0</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="N9" s="7"/>
       <c r="O9" s="7"/>
       <c r="P9" s="7"/>
     </row>
     <row r="10" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="H10" s="8" t="s">
-        <v>78</v>
+      <c r="H10" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="I10" s="7"/>
       <c r="J10" s="8" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="K10" s="7"/>
       <c r="L10" s="9">
         <v>0</v>
       </c>
       <c r="M10" s="6" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="N10" s="7"/>
       <c r="O10" s="7"/>
@@ -1122,18 +1178,20 @@
     </row>
     <row r="11" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H11" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="I11" s="7"/>
+        <v>83</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>84</v>
+      </c>
       <c r="J11" s="8" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="K11" s="7"/>
       <c r="L11" s="9">
         <v>0</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="N11" s="7"/>
       <c r="O11" s="7"/>
@@ -1141,91 +1199,107 @@
     </row>
     <row r="12" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H12" s="8" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="I12" s="7"/>
       <c r="J12" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="K12" s="7"/>
+        <v>67</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>87</v>
+      </c>
       <c r="L12" s="9">
         <v>0</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="N12" s="7"/>
       <c r="O12" s="7"/>
       <c r="P12" s="7"/>
     </row>
-    <row r="13" spans="1:16" ht="331.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H13" s="6" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="I13" s="7"/>
       <c r="J13" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>72</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="K13" s="7"/>
       <c r="L13" s="9">
         <v>0</v>
       </c>
       <c r="M13" s="8" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="N13" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="O13" s="6" t="s">
-        <v>74</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="O13" s="7"/>
       <c r="P13" s="7"/>
     </row>
     <row r="14" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H14" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="I14" s="7"/>
+        <v>89</v>
+      </c>
+      <c r="I14" s="8" t="s">
+        <v>90</v>
+      </c>
       <c r="J14" s="8" t="s">
-        <v>83</v>
+        <v>67</v>
       </c>
       <c r="K14" s="7"/>
       <c r="L14" s="9">
         <v>0</v>
       </c>
       <c r="M14" s="6" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="N14" s="7"/>
       <c r="O14" s="7"/>
       <c r="P14" s="7"/>
     </row>
-    <row r="15" spans="1:16" ht="409.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="H15" s="8" t="s">
-        <v>84</v>
+    <row r="15" spans="1:16" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="H15" s="6" t="s">
+        <v>91</v>
       </c>
       <c r="I15" s="7"/>
       <c r="J15" s="8" t="s">
-        <v>83</v>
+        <v>67</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="L15" s="9">
         <v>0</v>
       </c>
       <c r="M15" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="N15" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="O15" s="6" t="s">
-        <v>74</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="O15" s="7"/>
       <c r="P15" s="7"/>
+    </row>
+    <row r="16" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="H16" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="I16" s="7"/>
+      <c r="J16" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="K16" s="7"/>
+      <c r="L16" s="9">
+        <v>0</v>
+      </c>
+      <c r="M16" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="N16" s="7"/>
+      <c r="O16" s="7"/>
     </row>
     <row r="125" spans="13:13" x14ac:dyDescent="0.3">
       <c r="M125"/>
@@ -1309,7 +1383,7 @@
       <formula>NOT(ISERROR(SEARCH("acyl_3oxo",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I1 I16:I108">
+  <conditionalFormatting sqref="I1 I17:I108">
     <cfRule type="containsText" dxfId="13" priority="31" operator="containsText" text="acylcarnitine">
       <formula>NOT(ISERROR(SEARCH("acylcarnitine",I1)))</formula>
     </cfRule>
@@ -1344,6 +1418,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
modified metabolites additions file
</commit_message>
<xml_diff>
--- a/Tasks/Task_706_Gastrin_synthesis/metabolites_additions.xlsx
+++ b/Tasks/Task_706_Gastrin_synthesis/metabolites_additions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Desktop\Project Papers to Pathways\MSP_p3_2026_hormone_cytokine_task_creation\Tasks\Task_706_Gastrin_synthesis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emparsanjuliancano/Documents/GitHub/MSP_p3_2026_hormone_cytokine_task_creation/Tasks/Task_706_Gastrin_synthesis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F73AF981-065D-48D5-94C6-A4BC23EE05D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21778661-EBE7-DC4C-AB67-0F0C0E8BBC76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CD5DF94A-FED4-4ED9-B2C5-1CBFE42F25CF}"/>
+    <workbookView xWindow="3560" yWindow="740" windowWidth="23260" windowHeight="12460" xr2:uid="{CD5DF94A-FED4-4ED9-B2C5-1CBFE42F25CF}"/>
   </bookViews>
   <sheets>
     <sheet name="mets" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="94">
   <si>
     <t>action</t>
   </si>
@@ -237,13 +237,7 @@
     <t>r</t>
   </si>
   <si>
-    <t>P01189</t>
-  </si>
-  <si>
     <t>mg</t>
-  </si>
-  <si>
-    <t>P63267</t>
   </si>
   <si>
     <t>pre-pro-gastrin-1[c]</t>
@@ -933,19 +927,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D14686DA-B500-41AE-B187-0230B8D69B0A}">
   <dimension ref="A1:P268"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="7" max="7" width="22.44140625" customWidth="1"/>
-    <col min="8" max="8" width="28.109375" customWidth="1"/>
-    <col min="9" max="9" width="39.109375" customWidth="1"/>
-    <col min="10" max="10" width="11.44140625" style="2"/>
-    <col min="11" max="11" width="14.44140625" style="2" customWidth="1"/>
-    <col min="12" max="12" width="11.44140625" style="2"/>
-    <col min="13" max="13" width="32.109375" style="4" customWidth="1"/>
-    <col min="18" max="20" width="23.88671875" customWidth="1"/>
+    <col min="7" max="7" width="22.5" customWidth="1"/>
+    <col min="8" max="8" width="28.1640625" customWidth="1"/>
+    <col min="9" max="9" width="39.1640625" customWidth="1"/>
+    <col min="10" max="10" width="11.5" style="2"/>
+    <col min="11" max="11" width="14.5" style="2" customWidth="1"/>
+    <col min="12" max="12" width="11.5" style="2"/>
+    <col min="13" max="13" width="32.1640625" style="4" customWidth="1"/>
+    <col min="18" max="20" width="23.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -983,22 +977,22 @@
         <v>11</v>
       </c>
       <c r="N1" s="13" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="O1" s="13" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="145" thickBot="1" x14ac:dyDescent="0.25">
       <c r="H2" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I2" s="7"/>
       <c r="J2" s="8" t="s">
         <v>60</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L2" s="9">
         <v>0</v>
@@ -1007,23 +1001,23 @@
         <v>61</v>
       </c>
       <c r="N2" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="P2" s="7"/>
+    </row>
+    <row r="3" spans="1:16" ht="145" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="H3" s="6" t="s">
         <v>71</v>
-      </c>
-      <c r="O2" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="P2" s="7"/>
-    </row>
-    <row r="3" spans="1:16" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="H3" s="6" t="s">
-        <v>73</v>
       </c>
       <c r="I3" s="7"/>
       <c r="J3" s="8" t="s">
         <v>60</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L3" s="9">
         <v>0</v>
@@ -1032,16 +1026,16 @@
         <v>61</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O3" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="P3" s="7"/>
+    </row>
+    <row r="4" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="H4" s="6" t="s">
         <v>72</v>
-      </c>
-      <c r="P3" s="7"/>
-    </row>
-    <row r="4" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="H4" s="6" t="s">
-        <v>74</v>
       </c>
       <c r="I4" s="7"/>
       <c r="J4" s="8" t="s">
@@ -1058,9 +1052,9 @@
       <c r="O4" s="7"/>
       <c r="P4" s="7"/>
     </row>
-    <row r="5" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="H5" s="6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I5" s="7"/>
       <c r="J5" s="8" t="s">
@@ -1077,9 +1071,9 @@
       <c r="O5" s="7"/>
       <c r="P5" s="7"/>
     </row>
-    <row r="6" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="H6" s="6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I6" s="7"/>
       <c r="J6" s="8" t="s">
@@ -1096,9 +1090,9 @@
       <c r="O6" s="7"/>
       <c r="P6" s="7"/>
     </row>
-    <row r="7" spans="1:16" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="H7" s="10" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="I7" s="7"/>
       <c r="J7" s="8" t="s">
@@ -1111,22 +1105,20 @@
       <c r="M7" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="N7" s="8" t="s">
-        <v>66</v>
-      </c>
+      <c r="N7" s="8"/>
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
     </row>
-    <row r="8" spans="1:16" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" ht="33" thickBot="1" x14ac:dyDescent="0.25">
       <c r="H8" s="10" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="I8" s="7"/>
       <c r="J8" s="8" t="s">
         <v>65</v>
       </c>
       <c r="K8" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L8" s="9">
         <v>0</v>
@@ -1138,13 +1130,13 @@
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
     </row>
-    <row r="9" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="H9" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I9" s="7"/>
       <c r="J9" s="8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="K9" s="7"/>
       <c r="L9" s="9">
@@ -1157,13 +1149,13 @@
       <c r="O9" s="7"/>
       <c r="P9" s="7"/>
     </row>
-    <row r="10" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="H10" s="6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I10" s="7"/>
       <c r="J10" s="8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="K10" s="7"/>
       <c r="L10" s="9">
@@ -1176,15 +1168,15 @@
       <c r="O10" s="7"/>
       <c r="P10" s="7"/>
     </row>
-    <row r="11" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="H11" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="J11" s="8" t="s">
         <v>83</v>
-      </c>
-      <c r="I11" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>85</v>
       </c>
       <c r="K11" s="7"/>
       <c r="L11" s="9">
@@ -1197,16 +1189,16 @@
       <c r="O11" s="7"/>
       <c r="P11" s="7"/>
     </row>
-    <row r="12" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="H12" s="8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I12" s="7"/>
       <c r="J12" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K12" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L12" s="9">
         <v>0</v>
@@ -1218,13 +1210,13 @@
       <c r="O12" s="7"/>
       <c r="P12" s="7"/>
     </row>
-    <row r="13" spans="1:16" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="H13" s="6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I13" s="7"/>
       <c r="J13" s="8" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="K13" s="7"/>
       <c r="L13" s="9">
@@ -1233,21 +1225,19 @@
       <c r="M13" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="N13" s="8" t="s">
-        <v>66</v>
-      </c>
+      <c r="N13" s="8"/>
       <c r="O13" s="7"/>
       <c r="P13" s="7"/>
     </row>
-    <row r="14" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="H14" s="8" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K14" s="7"/>
       <c r="L14" s="9">
@@ -1260,16 +1250,16 @@
       <c r="O14" s="7"/>
       <c r="P14" s="7"/>
     </row>
-    <row r="15" spans="1:16" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" ht="129" thickBot="1" x14ac:dyDescent="0.25">
       <c r="H15" s="6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="I15" s="7"/>
       <c r="J15" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="L15" s="9">
         <v>0</v>
@@ -1277,19 +1267,17 @@
       <c r="M15" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="N15" s="8" t="s">
-        <v>68</v>
-      </c>
+      <c r="N15" s="8"/>
       <c r="O15" s="7"/>
       <c r="P15" s="7"/>
     </row>
-    <row r="16" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="H16" s="12" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="I16" s="7"/>
       <c r="J16" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K16" s="7"/>
       <c r="L16" s="9">
@@ -1301,67 +1289,67 @@
       <c r="N16" s="7"/>
       <c r="O16" s="7"/>
     </row>
-    <row r="125" spans="13:13" x14ac:dyDescent="0.3">
+    <row r="125" spans="13:13" x14ac:dyDescent="0.2">
       <c r="M125"/>
     </row>
-    <row r="126" spans="13:13" x14ac:dyDescent="0.3">
+    <row r="126" spans="13:13" x14ac:dyDescent="0.2">
       <c r="M126"/>
     </row>
-    <row r="145" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="145" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K145"/>
     </row>
-    <row r="146" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="146" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K146"/>
     </row>
-    <row r="147" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="147" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K147"/>
     </row>
-    <row r="148" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="148" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K148"/>
     </row>
-    <row r="149" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="149" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K149"/>
     </row>
-    <row r="150" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="150" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K150"/>
     </row>
-    <row r="151" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="151" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K151"/>
     </row>
-    <row r="152" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="152" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K152"/>
     </row>
-    <row r="153" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="153" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K153"/>
     </row>
-    <row r="259" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="259" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K259"/>
     </row>
-    <row r="260" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="260" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K260"/>
     </row>
-    <row r="261" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="261" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K261"/>
     </row>
-    <row r="262" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="262" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K262"/>
     </row>
-    <row r="263" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="263" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K263"/>
     </row>
-    <row r="264" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="264" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K264"/>
     </row>
-    <row r="265" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="265" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K265"/>
     </row>
-    <row r="266" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="266" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K266"/>
     </row>
-    <row r="267" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="267" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K267"/>
     </row>
-    <row r="268" spans="11:11" x14ac:dyDescent="0.3">
+    <row r="268" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K268"/>
     </row>
   </sheetData>
@@ -1425,13 +1413,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47C4FABE-BBAA-42F0-8C19-3F54C559520F}">
   <dimension ref="A1:C24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.44140625" customWidth="1"/>
-    <col min="2" max="2" width="26.109375" customWidth="1"/>
+    <col min="1" max="1" width="21.5" customWidth="1"/>
+    <col min="2" max="2" width="26.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -1439,7 +1427,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
@@ -1448,7 +1436,7 @@
       </c>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
@@ -1457,7 +1445,7 @@
       </c>
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>18</v>
       </c>
@@ -1466,7 +1454,7 @@
       </c>
       <c r="C4" s="1"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
@@ -1475,7 +1463,7 @@
       </c>
       <c r="C5" s="1"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
@@ -1484,7 +1472,7 @@
       </c>
       <c r="C6" s="1"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>24</v>
       </c>
@@ -1493,7 +1481,7 @@
       </c>
       <c r="C7" s="1"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>26</v>
       </c>
@@ -1502,7 +1490,7 @@
       </c>
       <c r="C8" s="1"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>28</v>
       </c>
@@ -1511,7 +1499,7 @@
       </c>
       <c r="C9" s="1"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>30</v>
       </c>
@@ -1520,7 +1508,7 @@
       </c>
       <c r="C10" s="1"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>32</v>
       </c>
@@ -1529,7 +1517,7 @@
       </c>
       <c r="C11" s="1"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>34</v>
       </c>
@@ -1538,7 +1526,7 @@
       </c>
       <c r="C12" s="1"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>36</v>
       </c>
@@ -1547,7 +1535,7 @@
       </c>
       <c r="C13" s="1"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>38</v>
       </c>
@@ -1556,7 +1544,7 @@
       </c>
       <c r="C14" s="1"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>40</v>
       </c>
@@ -1565,7 +1553,7 @@
       </c>
       <c r="C15" s="1"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>42</v>
       </c>
@@ -1574,7 +1562,7 @@
       </c>
       <c r="C16" s="1"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>44</v>
       </c>
@@ -1583,7 +1571,7 @@
       </c>
       <c r="C17" s="1"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>46</v>
       </c>
@@ -1592,7 +1580,7 @@
       </c>
       <c r="C18" s="1"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>48</v>
       </c>
@@ -1601,7 +1589,7 @@
       </c>
       <c r="C19" s="1"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>50</v>
       </c>
@@ -1610,7 +1598,7 @@
       </c>
       <c r="C20" s="1"/>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>52</v>
       </c>
@@ -1619,7 +1607,7 @@
       </c>
       <c r="C21" s="1"/>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>54</v>
       </c>
@@ -1628,7 +1616,7 @@
       </c>
       <c r="C22" s="1"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>56</v>
       </c>
@@ -1637,7 +1625,7 @@
       </c>
       <c r="C23" s="1"/>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>58</v>
       </c>

</xml_diff>